<commit_message>
🔒 [FULL] Daily chip data 2026-05-22 00:34
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-05-21.xlsx
+++ b/data/reports/chip_radar_2026-05-21.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00_ ;[Red]\-0.00\ "/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +39,12 @@
     <font>
       <name val="新細明體"/>
       <color rgb="FFFF0000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="新細明體"/>
+      <i val="1"/>
+      <color rgb="FF808080"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -62,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -80,6 +86,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -9108,7 +9117,7 @@
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>創意(3443) ▲9.99%</t>
+          <t>創意(3443)</t>
         </is>
       </c>
       <c r="E244" s="3" t="n">
@@ -9140,7 +9149,7 @@
     <row r="245" ht="16.5" customHeight="1">
       <c r="D245" s="2" t="inlineStr">
         <is>
-          <t>凱美(2375) ▲9.87%</t>
+          <t>凱美(2375)</t>
         </is>
       </c>
       <c r="E245" s="3" t="n">
@@ -9172,7 +9181,7 @@
     <row r="246" ht="16.5" customHeight="1">
       <c r="D246" s="2" t="inlineStr">
         <is>
-          <t>台燿(6274) ▲9.96%</t>
+          <t>台燿(6274)</t>
         </is>
       </c>
       <c r="E246" s="3" t="n">
@@ -9204,7 +9213,7 @@
     <row r="247" ht="16.5" customHeight="1">
       <c r="D247" s="2" t="inlineStr">
         <is>
-          <t>凌陽(2401) ▲9.85%</t>
+          <t>凌陽(2401)</t>
         </is>
       </c>
       <c r="E247" s="3" t="n">
@@ -9234,7 +9243,11 @@
       </c>
     </row>
     <row r="248" ht="16.5" customHeight="1">
-      <c r="D248" s="2" t="n"/>
+      <c r="D248" s="7" t="inlineStr">
+        <is>
+          <t>⚪ 今日漲停僅 4 檔</t>
+        </is>
+      </c>
       <c r="E248" s="3" t="n"/>
       <c r="F248" s="3" t="n"/>
       <c r="G248" s="3" t="n"/>
@@ -9369,7 +9382,7 @@
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>聯發科(2454) ▲9.91%</t>
+          <t>聯發科(2454)</t>
         </is>
       </c>
       <c r="E255" s="3" t="n">
@@ -9401,7 +9414,7 @@
     <row r="256" ht="16.5" customHeight="1">
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>群創(3481) ▲9.88%</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E256" s="3" t="n">
@@ -9433,7 +9446,7 @@
     <row r="257" ht="16.5" customHeight="1">
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>瑞軒(2489) ▲9.99%</t>
+          <t>瑞軒(2489)</t>
         </is>
       </c>
       <c r="E257" s="3" t="n">
@@ -9465,7 +9478,7 @@
     <row r="258" ht="16.5" customHeight="1">
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t>創意(3443) ▲9.99%</t>
+          <t>創意(3443)</t>
         </is>
       </c>
       <c r="E258" s="3" t="n">
@@ -9497,7 +9510,7 @@
     <row r="259" ht="16.5" customHeight="1">
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>欣興(3037) ▲9.96%</t>
+          <t>欣興(3037)</t>
         </is>
       </c>
       <c r="E259" s="3" t="n">
@@ -9529,7 +9542,7 @@
     <row r="260" ht="16.5" customHeight="1">
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>國巨*(2327) ▲10.0%</t>
+          <t>國巨*(2327)</t>
         </is>
       </c>
       <c r="E260" s="3" t="n">
@@ -9561,7 +9574,7 @@
     <row r="261" ht="16.5" customHeight="1">
       <c r="D261" s="2" t="inlineStr">
         <is>
-          <t>景碩(3189) ▲9.92%</t>
+          <t>景碩(3189)</t>
         </is>
       </c>
       <c r="E261" s="3" t="n">
@@ -9593,7 +9606,7 @@
     <row r="262" ht="16.5" customHeight="1">
       <c r="D262" s="2" t="inlineStr">
         <is>
-          <t>矽力*-KY(6415) ▲9.86%</t>
+          <t>矽力*-KY(6415)</t>
         </is>
       </c>
       <c r="E262" s="3" t="n">
@@ -9625,7 +9638,7 @@
     <row r="263" ht="16.5" customHeight="1">
       <c r="D263" s="2" t="inlineStr">
         <is>
-          <t>凌陽(2401) ▲9.85%</t>
+          <t>凌陽(2401)</t>
         </is>
       </c>
       <c r="E263" s="3" t="n">
@@ -9657,7 +9670,7 @@
     <row r="264" ht="16.5" customHeight="1">
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>彩晶(6116) ▲9.64%</t>
+          <t>彩晶(6116)</t>
         </is>
       </c>
       <c r="E264" s="3" t="n">
@@ -9756,7 +9769,7 @@
       </c>
       <c r="D266" s="2" t="inlineStr">
         <is>
-          <t>國巨*(2327) ▲10.0%</t>
+          <t>國巨*(2327)</t>
         </is>
       </c>
       <c r="E266" s="3" t="n">
@@ -9788,7 +9801,7 @@
     <row r="267" ht="16.5" customHeight="1">
       <c r="D267" s="2" t="inlineStr">
         <is>
-          <t>欣興(3037) ▲9.96%</t>
+          <t>欣興(3037)</t>
         </is>
       </c>
       <c r="E267" s="3" t="n">
@@ -9820,7 +9833,7 @@
     <row r="268" ht="16.5" customHeight="1">
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>創意(3443) ▲9.99%</t>
+          <t>創意(3443)</t>
         </is>
       </c>
       <c r="E268" s="3" t="n">
@@ -9852,7 +9865,7 @@
     <row r="269" ht="16.5" customHeight="1">
       <c r="D269" s="2" t="inlineStr">
         <is>
-          <t>群創(3481) ▲9.88%</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E269" s="3" t="n">
@@ -9884,7 +9897,7 @@
     <row r="270" ht="16.5" customHeight="1">
       <c r="D270" s="2" t="inlineStr">
         <is>
-          <t>景碩(3189) ▲9.92%</t>
+          <t>景碩(3189)</t>
         </is>
       </c>
       <c r="E270" s="3" t="n">
@@ -9916,7 +9929,7 @@
     <row r="271" ht="16.5" customHeight="1">
       <c r="D271" s="2" t="inlineStr">
         <is>
-          <t>矽力*-KY(6415) ▲9.86%</t>
+          <t>矽力*-KY(6415)</t>
         </is>
       </c>
       <c r="E271" s="3" t="n">
@@ -9948,7 +9961,7 @@
     <row r="272" ht="16.5" customHeight="1">
       <c r="D272" s="2" t="inlineStr">
         <is>
-          <t>瑞軒(2489) ▲9.99%</t>
+          <t>瑞軒(2489)</t>
         </is>
       </c>
       <c r="E272" s="3" t="n">
@@ -9980,7 +9993,7 @@
     <row r="273" ht="16.5" customHeight="1">
       <c r="D273" s="2" t="inlineStr">
         <is>
-          <t>誠美材(4960) ▲9.95%</t>
+          <t>誠美材(4960)</t>
         </is>
       </c>
       <c r="E273" s="3" t="n">
@@ -10012,7 +10025,7 @@
     <row r="274" ht="16.5" customHeight="1">
       <c r="D274" s="2" t="inlineStr">
         <is>
-          <t>中砂(1560) ▲9.85%</t>
+          <t>中砂(1560)</t>
         </is>
       </c>
       <c r="E274" s="3" t="n">
@@ -10044,7 +10057,7 @@
     <row r="275" ht="16.5" customHeight="1">
       <c r="D275" s="2" t="inlineStr">
         <is>
-          <t>雷科(6207) ▲9.91%</t>
+          <t>雷科(6207)</t>
         </is>
       </c>
       <c r="E275" s="3" t="n">
@@ -13269,7 +13282,7 @@
       </c>
       <c r="D365" s="2" t="inlineStr">
         <is>
-          <t>景碩(3189) ▲9.92%</t>
+          <t>景碩(3189)</t>
         </is>
       </c>
       <c r="E365" s="3" t="n">
@@ -13301,7 +13314,7 @@
     <row r="366" ht="16.5" customHeight="1">
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>欣興(3037) ▲9.96%</t>
+          <t>欣興(3037)</t>
         </is>
       </c>
       <c r="E366" s="3" t="n">
@@ -13333,7 +13346,7 @@
     <row r="367" ht="16.5" customHeight="1">
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>晶呈科技(4768) ▲9.99%</t>
+          <t>晶呈科技(4768)</t>
         </is>
       </c>
       <c r="E367" s="3" t="n">
@@ -13365,7 +13378,7 @@
     <row r="368" ht="16.5" customHeight="1">
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>國巨*(2327) ▲10.0%</t>
+          <t>國巨*(2327)</t>
         </is>
       </c>
       <c r="E368" s="3" t="n">
@@ -13397,7 +13410,7 @@
     <row r="369" ht="16.5" customHeight="1">
       <c r="D369" s="2" t="inlineStr">
         <is>
-          <t>新應材(4749) ▲9.66%</t>
+          <t>新應材(4749)</t>
         </is>
       </c>
       <c r="E369" s="3" t="n">
@@ -13429,7 +13442,7 @@
     <row r="370" ht="16.5" customHeight="1">
       <c r="D370" s="2" t="inlineStr">
         <is>
-          <t>益登(3048) ▲9.89%</t>
+          <t>益登(3048)</t>
         </is>
       </c>
       <c r="E370" s="3" t="n">
@@ -13461,7 +13474,7 @@
     <row r="371" ht="16.5" customHeight="1">
       <c r="D371" s="2" t="inlineStr">
         <is>
-          <t>波若威(3163) ▲9.77%</t>
+          <t>波若威(3163)</t>
         </is>
       </c>
       <c r="E371" s="3" t="n">
@@ -13493,7 +13506,7 @@
     <row r="372" ht="16.5" customHeight="1">
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t>牧德(3563) ▲9.89%</t>
+          <t>牧德(3563)</t>
         </is>
       </c>
       <c r="E372" s="3" t="n">
@@ -13525,7 +13538,7 @@
     <row r="373" ht="16.5" customHeight="1">
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t>凱美(2375) ▲9.87%</t>
+          <t>凱美(2375)</t>
         </is>
       </c>
       <c r="E373" s="3" t="n">
@@ -13557,7 +13570,7 @@
     <row r="374" ht="16.5" customHeight="1">
       <c r="D374" s="2" t="inlineStr">
         <is>
-          <t>有成精密(4949) ▲9.97%</t>
+          <t>有成精密(4949)</t>
         </is>
       </c>
       <c r="E374" s="3" t="n">
@@ -13666,7 +13679,7 @@
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t>聯發科(2454) ▲9.91%</t>
+          <t>聯發科(2454)</t>
         </is>
       </c>
       <c r="E376" s="3" t="n">
@@ -13698,7 +13711,7 @@
     <row r="377" ht="16.5" customHeight="1">
       <c r="D377" s="2" t="inlineStr">
         <is>
-          <t>瑞軒(2489) ▲9.99%</t>
+          <t>瑞軒(2489)</t>
         </is>
       </c>
       <c r="E377" s="3" t="n">
@@ -13730,7 +13743,7 @@
     <row r="378" ht="16.5" customHeight="1">
       <c r="D378" s="2" t="inlineStr">
         <is>
-          <t>單井(3490) ▲10.0%</t>
+          <t>單井(3490)</t>
         </is>
       </c>
       <c r="E378" s="3" t="n">
@@ -13762,7 +13775,7 @@
     <row r="379" ht="16.5" customHeight="1">
       <c r="D379" s="2" t="inlineStr">
         <is>
-          <t>創意(3443) ▲9.99%</t>
+          <t>創意(3443)</t>
         </is>
       </c>
       <c r="E379" s="3" t="n">
@@ -13794,7 +13807,7 @@
     <row r="380" ht="16.5" customHeight="1">
       <c r="D380" s="2" t="inlineStr">
         <is>
-          <t>新唐(4919) ▲10.0%</t>
+          <t>新唐(4919)</t>
         </is>
       </c>
       <c r="E380" s="3" t="n">
@@ -13826,7 +13839,7 @@
     <row r="381" ht="16.5" customHeight="1">
       <c r="D381" s="2" t="inlineStr">
         <is>
-          <t>嘉晶(3016) ▲10.0%</t>
+          <t>嘉晶(3016)</t>
         </is>
       </c>
       <c r="E381" s="3" t="n">
@@ -13858,7 +13871,7 @@
     <row r="382" ht="16.5" customHeight="1">
       <c r="D382" s="2" t="inlineStr">
         <is>
-          <t>合晶(6182) ▲9.84%</t>
+          <t>合晶(6182)</t>
         </is>
       </c>
       <c r="E382" s="3" t="n">
@@ -13890,7 +13903,7 @@
     <row r="383" ht="16.5" customHeight="1">
       <c r="D383" s="2" t="inlineStr">
         <is>
-          <t>牧德(3563) ▲9.89%</t>
+          <t>牧德(3563)</t>
         </is>
       </c>
       <c r="E383" s="3" t="n">
@@ -13922,7 +13935,7 @@
     <row r="384" ht="16.5" customHeight="1">
       <c r="D384" s="2" t="inlineStr">
         <is>
-          <t>堡達(3537) ▲9.86%</t>
+          <t>堡達(3537)</t>
         </is>
       </c>
       <c r="E384" s="3" t="n">
@@ -13954,7 +13967,7 @@
     <row r="385" ht="16.5" customHeight="1">
       <c r="D385" s="2" t="inlineStr">
         <is>
-          <t>亞泰金屬(6727) ▲9.97%</t>
+          <t>亞泰金屬(6727)</t>
         </is>
       </c>
       <c r="E385" s="3" t="n">
@@ -14053,7 +14066,7 @@
       </c>
       <c r="D387" s="2" t="inlineStr">
         <is>
-          <t>敬鵬(2355) ▲9.98%</t>
+          <t>敬鵬(2355)</t>
         </is>
       </c>
       <c r="E387" s="3" t="n">
@@ -14085,7 +14098,7 @@
     <row r="388" ht="16.5" customHeight="1">
       <c r="D388" s="2" t="inlineStr">
         <is>
-          <t>台表科(6278) ▲9.85%</t>
+          <t>台表科(6278)</t>
         </is>
       </c>
       <c r="E388" s="3" t="n">
@@ -14117,7 +14130,7 @@
     <row r="389" ht="16.5" customHeight="1">
       <c r="D389" s="2" t="inlineStr">
         <is>
-          <t>日電貿(3090) ▲9.8%</t>
+          <t>日電貿(3090)</t>
         </is>
       </c>
       <c r="E389" s="3" t="n">
@@ -14149,7 +14162,7 @@
     <row r="390" ht="16.5" customHeight="1">
       <c r="D390" s="2" t="inlineStr">
         <is>
-          <t>奇鈦科(3430) ▲9.78%</t>
+          <t>奇鈦科(3430)</t>
         </is>
       </c>
       <c r="E390" s="3" t="n">
@@ -14181,7 +14194,7 @@
     <row r="391" ht="16.5" customHeight="1">
       <c r="D391" s="2" t="inlineStr">
         <is>
-          <t>聯友金屬-創(7610) ▲9.82%</t>
+          <t>聯友金屬-創(7610)</t>
         </is>
       </c>
       <c r="E391" s="3" t="n">
@@ -14213,7 +14226,7 @@
     <row r="392" ht="16.5" customHeight="1">
       <c r="D392" s="2" t="inlineStr">
         <is>
-          <t>澤米(6742) ▲9.98%</t>
+          <t>澤米(6742)</t>
         </is>
       </c>
       <c r="E392" s="3" t="n">
@@ -14245,7 +14258,7 @@
     <row r="393" ht="16.5" customHeight="1">
       <c r="D393" s="2" t="inlineStr">
         <is>
-          <t>亞泰金屬(6727) ▲9.97%</t>
+          <t>亞泰金屬(6727)</t>
         </is>
       </c>
       <c r="E393" s="3" t="n">
@@ -14277,7 +14290,7 @@
     <row r="394" ht="16.5" customHeight="1">
       <c r="D394" s="2" t="inlineStr">
         <is>
-          <t>華新科(2492) ▲9.92%</t>
+          <t>華新科(2492)</t>
         </is>
       </c>
       <c r="E394" s="3" t="n">
@@ -14309,7 +14322,7 @@
     <row r="395" ht="16.5" customHeight="1">
       <c r="D395" s="2" t="inlineStr">
         <is>
-          <t>泰藝(8289) ▲9.95%</t>
+          <t>泰藝(8289)</t>
         </is>
       </c>
       <c r="E395" s="3" t="n">
@@ -14341,7 +14354,7 @@
     <row r="396" ht="16.5" customHeight="1">
       <c r="D396" s="2" t="inlineStr">
         <is>
-          <t>凱美(2375) ▲9.87%</t>
+          <t>凱美(2375)</t>
         </is>
       </c>
       <c r="E396" s="3" t="n">
@@ -14440,7 +14453,7 @@
       </c>
       <c r="D398" s="2" t="inlineStr">
         <is>
-          <t>同欣電(6271) ▲9.87%</t>
+          <t>同欣電(6271)</t>
         </is>
       </c>
       <c r="E398" s="3" t="n">
@@ -14472,7 +14485,7 @@
     <row r="399" ht="16.5" customHeight="1">
       <c r="D399" s="2" t="inlineStr">
         <is>
-          <t>鴻勁(7769) ▲9.96%</t>
+          <t>鴻勁(7769)</t>
         </is>
       </c>
       <c r="E399" s="3" t="n">
@@ -14504,7 +14517,7 @@
     <row r="400" ht="16.5" customHeight="1">
       <c r="D400" s="2" t="inlineStr">
         <is>
-          <t>九暘(8040) ▲9.93%</t>
+          <t>九暘(8040)</t>
         </is>
       </c>
       <c r="E400" s="3" t="n">
@@ -14534,7 +14547,11 @@
       </c>
     </row>
     <row r="401" ht="16.5" customHeight="1">
-      <c r="D401" s="2" t="n"/>
+      <c r="D401" s="7" t="inlineStr">
+        <is>
+          <t>⚪ 今日漲停僅 3 檔</t>
+        </is>
+      </c>
       <c r="E401" s="3" t="n"/>
       <c r="F401" s="3" t="n"/>
       <c r="G401" s="3" t="n"/>
@@ -14690,7 +14707,7 @@
       </c>
       <c r="D409" s="2" t="inlineStr">
         <is>
-          <t>力成(6239) ▲9.81%</t>
+          <t>力成(6239)</t>
         </is>
       </c>
       <c r="E409" s="3" t="n">
@@ -14722,7 +14739,7 @@
     <row r="410" ht="16.5" customHeight="1">
       <c r="D410" s="2" t="inlineStr">
         <is>
-          <t>國巨*(2327) ▲10.0%</t>
+          <t>國巨*(2327)</t>
         </is>
       </c>
       <c r="E410" s="3" t="n">
@@ -14754,7 +14771,7 @@
     <row r="411" ht="16.5" customHeight="1">
       <c r="D411" s="2" t="inlineStr">
         <is>
-          <t>欣興(3037) ▲9.96%</t>
+          <t>欣興(3037)</t>
         </is>
       </c>
       <c r="E411" s="3" t="n">
@@ -14786,7 +14803,7 @@
     <row r="412" ht="16.5" customHeight="1">
       <c r="D412" s="2" t="inlineStr">
         <is>
-          <t>新唐(4919) ▲10.0%</t>
+          <t>新唐(4919)</t>
         </is>
       </c>
       <c r="E412" s="3" t="n">
@@ -14818,7 +14835,7 @@
     <row r="413" ht="16.5" customHeight="1">
       <c r="D413" s="2" t="inlineStr">
         <is>
-          <t>群創(3481) ▲9.88%</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E413" s="3" t="n">
@@ -14850,7 +14867,7 @@
     <row r="414" ht="16.5" customHeight="1">
       <c r="D414" s="2" t="inlineStr">
         <is>
-          <t>台表科(6278) ▲9.85%</t>
+          <t>台表科(6278)</t>
         </is>
       </c>
       <c r="E414" s="3" t="n">
@@ -14882,7 +14899,7 @@
     <row r="415" ht="16.5" customHeight="1">
       <c r="D415" s="2" t="inlineStr">
         <is>
-          <t>信錦(1582) ▲9.81%</t>
+          <t>信錦(1582)</t>
         </is>
       </c>
       <c r="E415" s="3" t="n">
@@ -14914,7 +14931,7 @@
     <row r="416" ht="16.5" customHeight="1">
       <c r="D416" s="2" t="inlineStr">
         <is>
-          <t>合一(4743) ▲10.0%</t>
+          <t>合一(4743)</t>
         </is>
       </c>
       <c r="E416" s="3" t="n">
@@ -14946,7 +14963,7 @@
     <row r="417" ht="16.5" customHeight="1">
       <c r="D417" s="2" t="inlineStr">
         <is>
-          <t>三集瑞-KY(6862) ▲9.94%</t>
+          <t>三集瑞-KY(6862)</t>
         </is>
       </c>
       <c r="E417" s="3" t="n">
@@ -14978,7 +14995,7 @@
     <row r="418" ht="16.5" customHeight="1">
       <c r="D418" s="2" t="inlineStr">
         <is>
-          <t>環球晶(6488) ▲9.87%</t>
+          <t>環球晶(6488)</t>
         </is>
       </c>
       <c r="E418" s="3" t="n">
@@ -15077,7 +15094,7 @@
       </c>
       <c r="D420" s="2" t="inlineStr">
         <is>
-          <t>科嶠(4542) ▲9.96%</t>
+          <t>科嶠(4542)</t>
         </is>
       </c>
       <c r="E420" s="3" t="n">
@@ -15109,7 +15126,7 @@
     <row r="421" ht="16.5" customHeight="1">
       <c r="D421" s="2" t="inlineStr">
         <is>
-          <t>華新科(2492) ▲9.92%</t>
+          <t>華新科(2492)</t>
         </is>
       </c>
       <c r="E421" s="3" t="n">
@@ -15141,7 +15158,7 @@
     <row r="422" ht="16.5" customHeight="1">
       <c r="D422" s="2" t="inlineStr">
         <is>
-          <t>台燿(6274) ▲9.96%</t>
+          <t>台燿(6274)</t>
         </is>
       </c>
       <c r="E422" s="3" t="n">
@@ -15173,7 +15190,7 @@
     <row r="423" ht="16.5" customHeight="1">
       <c r="D423" s="2" t="inlineStr">
         <is>
-          <t>波若威(3163) ▲9.77%</t>
+          <t>波若威(3163)</t>
         </is>
       </c>
       <c r="E423" s="3" t="n">
@@ -15205,7 +15222,7 @@
     <row r="424" ht="16.5" customHeight="1">
       <c r="D424" s="2" t="inlineStr">
         <is>
-          <t>同欣電(6271) ▲9.87%</t>
+          <t>同欣電(6271)</t>
         </is>
       </c>
       <c r="E424" s="3" t="n">
@@ -15237,7 +15254,7 @@
     <row r="425" ht="16.5" customHeight="1">
       <c r="D425" s="2" t="inlineStr">
         <is>
-          <t>群創(3481) ▲9.88%</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E425" s="3" t="n">
@@ -15269,7 +15286,7 @@
     <row r="426" ht="16.5" customHeight="1">
       <c r="D426" s="2" t="inlineStr">
         <is>
-          <t>矽力*-KY(6415) ▲9.86%</t>
+          <t>矽力*-KY(6415)</t>
         </is>
       </c>
       <c r="E426" s="3" t="n">
@@ -15301,7 +15318,7 @@
     <row r="427" ht="16.5" customHeight="1">
       <c r="D427" s="2" t="inlineStr">
         <is>
-          <t>台表科(6278) ▲9.85%</t>
+          <t>台表科(6278)</t>
         </is>
       </c>
       <c r="E427" s="3" t="n">
@@ -15333,7 +15350,7 @@
     <row r="428" ht="16.5" customHeight="1">
       <c r="D428" s="2" t="inlineStr">
         <is>
-          <t>新應材(4749) ▲9.66%</t>
+          <t>新應材(4749)</t>
         </is>
       </c>
       <c r="E428" s="3" t="n">
@@ -15365,7 +15382,7 @@
     <row r="429" ht="16.5" customHeight="1">
       <c r="D429" s="2" t="inlineStr">
         <is>
-          <t>漢磊(3707) ▲9.89%</t>
+          <t>漢磊(3707)</t>
         </is>
       </c>
       <c r="E429" s="3" t="n">

</xml_diff>